<commit_message>
tests: rename hyperlink test and cover file:// links
Rename issue_360_hyperlinks_xlsx to test_hyperlinks_xlsx and extend the
fixture with file:// hyperlink cases (local file, relative/absolute paths,
and links carrying an in-file anchor via location).
</commit_message>
<xml_diff>
--- a/tests/hyperlinks.xlsx
+++ b/tests/hyperlinks.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,6 +445,41 @@
       <c r="A3" t="inlineStr">
         <is>
           <t>go to other sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>book2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>sales book2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>temp book1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>book2 sheet1 a1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>sales data range</t>
         </is>
       </c>
     </row>
@@ -457,6 +492,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1:C2" tooltip="Email Foo" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" tooltip="Rust homepage" display="Rust Programming Language" r:id="rId3"/>
     <hyperlink ref="A3" location="'Sheet2'!B5" display="Sheet2 B5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" location="Sheet1!A1" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" location="'Sales Data'!A1:G5" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>